<commit_message>
fix(faqs): two-column layout, accent underline, source-parity accordion
Match the FAQs page to source:
- restructure the FAQ importer into a single two-column `faq-aside` section:
  FAQ heading + hero + intro + accordion in the left column, "Need more help?"
  contact block in a right aside (was one flat column with the aside pushed to
  the bottom). Section Metadata is emitted explicitly since a one-section page
  gets no <hr>-anchored style otherwise.
- styles.css: .section.faq-aside grid (2fr/1fr at >=900px, stacked mobile,
  top-aligned); hero constrained to the content column; intro justified with
  larger line-height; serif "Need more help?" aside heading; yellow underline
  under the FAQs H1 (via the existing yellow-underline style).
- accordion.css: plus/minus toggle icon (was chevron); bottom-divider-only rows
  (removed box borders + open yellow top border); uppercase bold sans-serif
  smaller question labels.

All FAQ text/links preserved (incl. source "WKDN" typo).
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-faqs.report.xlsx
+++ b/tools/importer/reports/import-faqs.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="209">
   <si>
     <t>_reportFile</t>
   </si>
@@ -61,7 +61,7 @@
     <t>home</t>
   </si>
   <si>
-    <t>2026-09-13T22:53:37.503Z</t>
+    <t>2026-09-18T10:56:49.249Z</t>
   </si>
   <si>
     <t>WKND Adventures and Travel</t>
@@ -70,10 +70,31 @@
     <t>https://wknd.site/us/en.html</t>
   </si>
   <si>
+    <t>us/en/about-us.report.json</t>
+  </si>
+  <si>
+    <t>["cards-people","cards-people","cards-people","cards-people","cards-people","cards-people","cards-people"]</t>
+  </si>
+  <si>
+    <t>us/en/about-us</t>
+  </si>
+  <si>
+    <t>about-us</t>
+  </si>
+  <si>
+    <t>2026-09-14T18:16:29.575Z</t>
+  </si>
+  <si>
+    <t>About Us</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/about-us.html</t>
+  </si>
+  <si>
     <t>us/en/adventures.report.json</t>
   </si>
   <si>
-    <t>["carousel","adventure-list","adventure-list","adventure-list","adventure-list","adventure-list","adventure-list"]</t>
+    <t>["carousel","cards","cards","cards","cards","cards","cards"]</t>
   </si>
   <si>
     <t>us/en/adventures</t>
@@ -82,7 +103,7 @@
     <t>adventures-landing</t>
   </si>
   <si>
-    <t>2026-09-14T11:48:04.413Z</t>
+    <t>2026-09-18T13:11:34.222Z</t>
   </si>
   <si>
     <t>Adventures</t>
@@ -103,7 +124,7 @@
     <t>faqs</t>
   </si>
   <si>
-    <t>2026-09-14T15:15:52.540Z</t>
+    <t>2026-09-21T10:43:26.907Z</t>
   </si>
   <si>
     <t>FAQs</t>
@@ -124,7 +145,7 @@
     <t>magazine</t>
   </si>
   <si>
-    <t>2026-09-14T12:11:58.324Z</t>
+    <t>2026-09-20T20:24:55.907Z</t>
   </si>
   <si>
     <t>Magazine</t>
@@ -134,6 +155,51 @@
   </si>
   <si>
     <t>us/en/adventures/bali-surf-camp.html.report.json</t>
+  </si>
+  <si>
+    <t xml:space="preserve">page.evaluate: Error: Failed to import page: metaBlock.querySelector is not a function
+    at eval (eval at evaluate (:290:30), &lt;anonymous&gt;:29:15)
+    at async &lt;anonymous&gt;:316:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">page.evaluate: Error: Failed to import page: metaBlock.querySelector is not a function
+    at eval (eval at evaluate (:290:30), &lt;anonymous&gt;:29:15)
+    at async &lt;anonymous&gt;:316:30
+    at processUrl (/home/node/.excat-marketplaces/excat-marketplace/excat/skills/excat-content-import/scripts/run-bulk-import.js:691:31)
+    at async main (/home/node/.excat-marketplaces/excat-marketplace/excat/skills/excat-content-import/scripts/run-bulk-import.js:954:22)</t>
+  </si>
+  <si>
+    <t>us/en/adventures/bali-surf-camp.html</t>
+  </si>
+  <si>
+    <t>failed</t>
+  </si>
+  <si>
+    <t>2026-09-14T18:41:29.034Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/bali-surf-camp.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/bali-surf-camp.report.json</t>
+  </si>
+  <si>
+    <t>["breadcrumb","carousel","columns","tabs"]</t>
+  </si>
+  <si>
+    <t>us/en/adventures/bali-surf-camp</t>
+  </si>
+  <si>
+    <t>adventures</t>
+  </si>
+  <si>
+    <t>2026-09-14T18:42:15.840Z</t>
+  </si>
+  <si>
+    <t>Bali Surf Camp</t>
+  </si>
+  <si>
+    <t>us/en/adventures/beervana-portland.html.report.json</t>
   </si>
   <si>
     <t xml:space="preserve">page.evaluate: Error: Failed to import page: metaBlock.append is not a function
@@ -148,39 +214,6 @@
     at async main (/home/node/.excat-marketplaces/excat-marketplace/excat/skills/excat-content-import/scripts/run-bulk-import.js:954:22)</t>
   </si>
   <si>
-    <t>us/en/adventures/bali-surf-camp.html</t>
-  </si>
-  <si>
-    <t>failed</t>
-  </si>
-  <si>
-    <t>2026-09-14T10:59:31.819Z</t>
-  </si>
-  <si>
-    <t>https://wknd.site/us/en/adventures/bali-surf-camp.html</t>
-  </si>
-  <si>
-    <t>us/en/adventures/bali-surf-camp.report.json</t>
-  </si>
-  <si>
-    <t>["breadcrumb","carousel","columns","tabs"]</t>
-  </si>
-  <si>
-    <t>us/en/adventures/bali-surf-camp</t>
-  </si>
-  <si>
-    <t>adventures</t>
-  </si>
-  <si>
-    <t>2026-09-14T11:00:09.445Z</t>
-  </si>
-  <si>
-    <t>Bali Surf Camp</t>
-  </si>
-  <si>
-    <t>us/en/adventures/beervana-portland.html.report.json</t>
-  </si>
-  <si>
     <t>us/en/adventures/beervana-portland.html</t>
   </si>
   <si>
@@ -196,7 +229,7 @@
     <t>us/en/adventures/beervana-portland</t>
   </si>
   <si>
-    <t>2026-09-14T11:00:15.307Z</t>
+    <t>2026-09-14T18:42:20.466Z</t>
   </si>
   <si>
     <t>Beervana in Portland</t>
@@ -220,7 +253,7 @@
     <t>us/en/adventures/climbing-new-zealand</t>
   </si>
   <si>
-    <t>2026-09-14T11:00:20.206Z</t>
+    <t>2026-09-14T18:42:26.387Z</t>
   </si>
   <si>
     <t>Climbing New Zealand</t>
@@ -244,7 +277,7 @@
     <t>us/en/adventures/colorado-rock-climbing</t>
   </si>
   <si>
-    <t>2026-09-14T11:00:24.848Z</t>
+    <t>2026-09-14T18:42:31.422Z</t>
   </si>
   <si>
     <t>Colorado Rock Climbing</t>
@@ -268,7 +301,7 @@
     <t>us/en/adventures/cycling-southern-utah</t>
   </si>
   <si>
-    <t>2026-09-14T11:00:31.131Z</t>
+    <t>2026-09-14T18:42:37.023Z</t>
   </si>
   <si>
     <t>Cycling Southern Utah</t>
@@ -292,7 +325,7 @@
     <t>us/en/adventures/cycling-tuscany</t>
   </si>
   <si>
-    <t>2026-09-14T11:00:34.811Z</t>
+    <t>2026-09-14T18:42:42.948Z</t>
   </si>
   <si>
     <t>Cycling Tuscany</t>
@@ -316,7 +349,7 @@
     <t>us/en/adventures/downhill-skiing-wyoming</t>
   </si>
   <si>
-    <t>2026-09-14T11:00:39.962Z</t>
+    <t>2026-09-14T18:42:47.711Z</t>
   </si>
   <si>
     <t>Downhill Skiing Wyoming</t>
@@ -340,7 +373,7 @@
     <t>us/en/adventures/gastronomic-marais-tour</t>
   </si>
   <si>
-    <t>2026-09-14T11:00:43.916Z</t>
+    <t>2026-09-14T18:42:53.912Z</t>
   </si>
   <si>
     <t>Gastronomic Marais Tour</t>
@@ -364,7 +397,7 @@
     <t>us/en/adventures/napa-wine-tasting</t>
   </si>
   <si>
-    <t>2026-09-14T11:00:50.670Z</t>
+    <t>2026-09-14T18:42:58.918Z</t>
   </si>
   <si>
     <t>Napa Wine Tasting</t>
@@ -388,7 +421,7 @@
     <t>us/en/adventures/riverside-camping-australia</t>
   </si>
   <si>
-    <t>2026-09-14T11:00:55.192Z</t>
+    <t>2026-09-14T18:43:04.684Z</t>
   </si>
   <si>
     <t>Riverside Camping</t>
@@ -412,7 +445,7 @@
     <t>us/en/adventures/ski-touring-mont-blanc</t>
   </si>
   <si>
-    <t>2026-09-14T11:00:59.840Z</t>
+    <t>2026-09-14T18:43:10.461Z</t>
   </si>
   <si>
     <t>Ski Touring Mont Blanc</t>
@@ -436,7 +469,7 @@
     <t>us/en/adventures/surf-camp-costa-rica</t>
   </si>
   <si>
-    <t>2026-09-14T11:01:04.096Z</t>
+    <t>2026-09-14T18:43:15.201Z</t>
   </si>
   <si>
     <t>Surf Camp in Costa Rica</t>
@@ -460,7 +493,7 @@
     <t>us/en/adventures/tahoe-skiing</t>
   </si>
   <si>
-    <t>2026-09-14T11:01:07.840Z</t>
+    <t>2026-09-14T18:43:19.845Z</t>
   </si>
   <si>
     <t>Tahoe Skiing</t>
@@ -484,7 +517,7 @@
     <t>us/en/adventures/west-coast-cycling</t>
   </si>
   <si>
-    <t>2026-09-14T11:01:12.189Z</t>
+    <t>2026-09-14T18:43:23.793Z</t>
   </si>
   <si>
     <t>West Coast Cycling</t>
@@ -508,7 +541,7 @@
     <t>us/en/adventures/whistler-mountain-biking</t>
   </si>
   <si>
-    <t>2026-09-14T11:01:17.884Z</t>
+    <t>2026-09-14T18:43:29.226Z</t>
   </si>
   <si>
     <t>Whistler Mountain Biking</t>
@@ -532,10 +565,91 @@
     <t>us/en/adventures/yosemite-backpacking</t>
   </si>
   <si>
-    <t>2026-09-14T11:01:22.539Z</t>
+    <t>2026-09-14T18:43:34.744Z</t>
   </si>
   <si>
     <t>Yosemite Backpacking</t>
+  </si>
+  <si>
+    <t>us/en/magazine/arctic-surfing.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/arctic-surfing</t>
+  </si>
+  <si>
+    <t>magazine-article</t>
+  </si>
+  <si>
+    <t>2026-09-21T01:37:01.549Z</t>
+  </si>
+  <si>
+    <t>Arctic Surfing</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/arctic-surfing.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine/guide-la-skateparks.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/guide-la-skateparks</t>
+  </si>
+  <si>
+    <t>skateparks-article</t>
+  </si>
+  <si>
+    <t>2026-09-21T00:41:38.123Z</t>
+  </si>
+  <si>
+    <t>Ultimate Guide to LA Skateparks</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/guide-la-skateparks.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine/san-diego-surf.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/san-diego-surf</t>
+  </si>
+  <si>
+    <t>2026-09-21T01:37:06.650Z</t>
+  </si>
+  <si>
+    <t>San Diego Surf Spots</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/san-diego-surf.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine/ski-touring.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/ski-touring</t>
+  </si>
+  <si>
+    <t>2026-09-21T01:37:12.865Z</t>
+  </si>
+  <si>
+    <t>Ski Touring</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/ski-touring.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine/western-australia.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/western-australia</t>
+  </si>
+  <si>
+    <t>2026-09-21T01:37:17.862Z</t>
+  </si>
+  <si>
+    <t>Western Australia</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/western-australia.html</t>
   </si>
 </sst>
 </file>
@@ -924,13 +1038,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="5" width="50" customWidth="1"/>
     <col min="7" max="7" width="20" customWidth="1"/>
     <col min="8" max="8" width="26" customWidth="1"/>
-    <col min="9" max="9" width="28" customWidth="1"/>
+    <col min="9" max="9" width="33" customWidth="1"/>
     <col min="10" max="10" width="50" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1099,28 +1213,28 @@
         <v>40</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="C6" t="s">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="D6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" t="s">
         <v>42</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" t="s">
         <v>43</v>
       </c>
-      <c r="F6" t="s">
+      <c r="H6" t="s">
         <v>44</v>
       </c>
-      <c r="G6" t="s">
-        <v>12</v>
-      </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>45</v>
-      </c>
-      <c r="I6" t="s">
-        <v>12</v>
       </c>
       <c r="J6" t="s">
         <v>46</v>
@@ -1131,991 +1245,1183 @@
         <v>47</v>
       </c>
       <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
         <v>48</v>
       </c>
-      <c r="C7" t="s">
-        <v>12</v>
-      </c>
       <c r="D7" t="s">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="E7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F7" t="s">
-        <v>14</v>
+        <v>51</v>
       </c>
       <c r="G7" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I7" t="s">
-        <v>52</v>
+        <v>12</v>
       </c>
       <c r="J7" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" t="s">
+        <v>56</v>
+      </c>
+      <c r="F8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" t="s">
+        <v>57</v>
+      </c>
+      <c r="H8" t="s">
+        <v>58</v>
+      </c>
+      <c r="I8" t="s">
+        <v>59</v>
+      </c>
+      <c r="J8" t="s">
         <v>53</v>
-      </c>
-      <c r="B8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" t="s">
-        <v>41</v>
-      </c>
-      <c r="D8" t="s">
-        <v>42</v>
-      </c>
-      <c r="E8" t="s">
-        <v>54</v>
-      </c>
-      <c r="F8" t="s">
-        <v>44</v>
-      </c>
-      <c r="G8" t="s">
-        <v>12</v>
-      </c>
-      <c r="H8" t="s">
-        <v>55</v>
-      </c>
-      <c r="I8" t="s">
-        <v>12</v>
-      </c>
-      <c r="J8" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B9" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C9" t="s">
-        <v>12</v>
+        <v>61</v>
       </c>
       <c r="D9" t="s">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="E9" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="F9" t="s">
-        <v>14</v>
+        <v>51</v>
       </c>
       <c r="G9" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H9" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I9" t="s">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="J9" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="B10" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="C10" t="s">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="D10" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="E10" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="F10" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="G10" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="H10" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="I10" t="s">
-        <v>12</v>
+        <v>69</v>
       </c>
       <c r="J10" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="B11" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C11" t="s">
-        <v>12</v>
+        <v>61</v>
       </c>
       <c r="D11" t="s">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="E11" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="F11" t="s">
-        <v>14</v>
+        <v>51</v>
       </c>
       <c r="G11" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H11" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="I11" t="s">
-        <v>68</v>
+        <v>12</v>
       </c>
       <c r="J11" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B12" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="C12" t="s">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="D12" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="E12" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="F12" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="G12" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="H12" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="I12" t="s">
-        <v>12</v>
+        <v>77</v>
       </c>
       <c r="J12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="B13" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>12</v>
+        <v>61</v>
       </c>
       <c r="D13" t="s">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="E13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="F13" t="s">
-        <v>14</v>
+        <v>51</v>
       </c>
       <c r="G13" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H13" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="I13" t="s">
-        <v>76</v>
+        <v>12</v>
       </c>
       <c r="J13" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="B14" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="C14" t="s">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="D14" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="E14" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="F14" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="G14" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="H14" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I14" t="s">
-        <v>12</v>
+        <v>85</v>
       </c>
       <c r="J14" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="B15" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C15" t="s">
-        <v>12</v>
+        <v>61</v>
       </c>
       <c r="D15" t="s">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="E15" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="F15" t="s">
-        <v>14</v>
+        <v>51</v>
       </c>
       <c r="G15" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H15" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="I15" t="s">
-        <v>84</v>
+        <v>12</v>
       </c>
       <c r="J15" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="B16" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="C16" t="s">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="D16" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="E16" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="F16" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="G16" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="H16" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="I16" t="s">
-        <v>12</v>
+        <v>93</v>
       </c>
       <c r="J16" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B17" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C17" t="s">
-        <v>12</v>
+        <v>61</v>
       </c>
       <c r="D17" t="s">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="E17" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="F17" t="s">
-        <v>14</v>
+        <v>51</v>
       </c>
       <c r="G17" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H17" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="I17" t="s">
-        <v>92</v>
+        <v>12</v>
       </c>
       <c r="J17" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="B18" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="C18" t="s">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="D18" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="E18" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="F18" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="G18" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="H18" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="I18" t="s">
-        <v>12</v>
+        <v>101</v>
       </c>
       <c r="J18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B19" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C19" t="s">
-        <v>12</v>
+        <v>61</v>
       </c>
       <c r="D19" t="s">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="E19" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="F19" t="s">
-        <v>14</v>
+        <v>51</v>
       </c>
       <c r="G19" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H19" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="I19" t="s">
-        <v>100</v>
+        <v>12</v>
       </c>
       <c r="J19" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="B20" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="C20" t="s">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="D20" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="E20" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="F20" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="G20" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="H20" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I20" t="s">
-        <v>12</v>
+        <v>109</v>
       </c>
       <c r="J20" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="B21" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C21" t="s">
-        <v>12</v>
+        <v>61</v>
       </c>
       <c r="D21" t="s">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="E21" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="F21" t="s">
-        <v>14</v>
+        <v>51</v>
       </c>
       <c r="G21" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H21" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="I21" t="s">
-        <v>108</v>
+        <v>12</v>
       </c>
       <c r="J21" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="B22" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="C22" t="s">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="D22" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="E22" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="F22" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="G22" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="H22" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="I22" t="s">
-        <v>12</v>
+        <v>117</v>
       </c>
       <c r="J22" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="B23" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C23" t="s">
-        <v>12</v>
+        <v>61</v>
       </c>
       <c r="D23" t="s">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="E23" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="F23" t="s">
-        <v>14</v>
+        <v>51</v>
       </c>
       <c r="G23" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H23" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="I23" t="s">
-        <v>116</v>
+        <v>12</v>
       </c>
       <c r="J23" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="B24" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="C24" t="s">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="D24" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="E24" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="F24" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="G24" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="H24" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="I24" t="s">
-        <v>12</v>
+        <v>125</v>
       </c>
       <c r="J24" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B25" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C25" t="s">
-        <v>12</v>
+        <v>61</v>
       </c>
       <c r="D25" t="s">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="E25" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="F25" t="s">
-        <v>14</v>
+        <v>51</v>
       </c>
       <c r="G25" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H25" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="I25" t="s">
-        <v>124</v>
+        <v>12</v>
       </c>
       <c r="J25" t="s">
-        <v>120</v>
+        <v>129</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B26" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="C26" t="s">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="D26" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="E26" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="F26" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="G26" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="H26" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="I26" t="s">
-        <v>12</v>
+        <v>133</v>
       </c>
       <c r="J26" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="B27" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C27" t="s">
-        <v>12</v>
+        <v>61</v>
       </c>
       <c r="D27" t="s">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="E27" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="F27" t="s">
-        <v>14</v>
+        <v>51</v>
       </c>
       <c r="G27" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H27" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="I27" t="s">
-        <v>132</v>
+        <v>12</v>
       </c>
       <c r="J27" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="B28" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="C28" t="s">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="D28" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="E28" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="F28" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="G28" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="H28" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="I28" t="s">
-        <v>12</v>
+        <v>141</v>
       </c>
       <c r="J28" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="B29" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C29" t="s">
-        <v>12</v>
+        <v>61</v>
       </c>
       <c r="D29" t="s">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="E29" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="F29" t="s">
-        <v>14</v>
+        <v>51</v>
       </c>
       <c r="G29" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H29" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="I29" t="s">
-        <v>140</v>
+        <v>12</v>
       </c>
       <c r="J29" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="B30" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="C30" t="s">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="D30" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="E30" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="F30" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="G30" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="H30" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="I30" t="s">
-        <v>12</v>
+        <v>149</v>
       </c>
       <c r="J30" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="B31" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C31" t="s">
-        <v>12</v>
+        <v>61</v>
       </c>
       <c r="D31" t="s">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="E31" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="F31" t="s">
-        <v>14</v>
+        <v>51</v>
       </c>
       <c r="G31" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H31" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="I31" t="s">
-        <v>148</v>
+        <v>12</v>
       </c>
       <c r="J31" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="B32" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="C32" t="s">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="D32" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="E32" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="F32" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="G32" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="H32" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="I32" t="s">
-        <v>12</v>
+        <v>157</v>
       </c>
       <c r="J32" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="B33" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C33" t="s">
-        <v>12</v>
+        <v>61</v>
       </c>
       <c r="D33" t="s">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="E33" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="F33" t="s">
-        <v>14</v>
+        <v>51</v>
       </c>
       <c r="G33" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H33" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="I33" t="s">
-        <v>156</v>
+        <v>12</v>
       </c>
       <c r="J33" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="B34" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="C34" t="s">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="D34" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="E34" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="F34" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="G34" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="H34" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="I34" t="s">
-        <v>12</v>
+        <v>165</v>
       </c>
       <c r="J34" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="B35" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C35" t="s">
-        <v>12</v>
+        <v>61</v>
       </c>
       <c r="D35" t="s">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="E35" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="F35" t="s">
-        <v>14</v>
+        <v>51</v>
       </c>
       <c r="G35" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H35" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="I35" t="s">
-        <v>164</v>
+        <v>12</v>
       </c>
       <c r="J35" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B36" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="C36" t="s">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="D36" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="E36" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="F36" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="G36" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="H36" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="I36" t="s">
-        <v>12</v>
+        <v>173</v>
       </c>
       <c r="J36" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="B37" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C37" t="s">
-        <v>12</v>
+        <v>61</v>
       </c>
       <c r="D37" t="s">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="E37" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="F37" t="s">
-        <v>14</v>
+        <v>51</v>
       </c>
       <c r="G37" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H37" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="I37" t="s">
-        <v>172</v>
+        <v>12</v>
       </c>
       <c r="J37" t="s">
-        <v>168</v>
+        <v>177</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>178</v>
+      </c>
+      <c r="B38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C38" t="s">
+        <v>12</v>
+      </c>
+      <c r="D38" t="s">
+        <v>12</v>
+      </c>
+      <c r="E38" t="s">
+        <v>179</v>
+      </c>
+      <c r="F38" t="s">
+        <v>14</v>
+      </c>
+      <c r="G38" t="s">
+        <v>57</v>
+      </c>
+      <c r="H38" t="s">
+        <v>180</v>
+      </c>
+      <c r="I38" t="s">
+        <v>181</v>
+      </c>
+      <c r="J38" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>182</v>
+      </c>
+      <c r="B39" t="s">
+        <v>12</v>
+      </c>
+      <c r="C39" t="s">
+        <v>12</v>
+      </c>
+      <c r="D39" t="s">
+        <v>12</v>
+      </c>
+      <c r="E39" t="s">
+        <v>183</v>
+      </c>
+      <c r="F39" t="s">
+        <v>14</v>
+      </c>
+      <c r="G39" t="s">
+        <v>184</v>
+      </c>
+      <c r="H39" t="s">
+        <v>185</v>
+      </c>
+      <c r="I39" t="s">
+        <v>186</v>
+      </c>
+      <c r="J39" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>188</v>
+      </c>
+      <c r="B40" t="s">
+        <v>12</v>
+      </c>
+      <c r="C40" t="s">
+        <v>12</v>
+      </c>
+      <c r="D40" t="s">
+        <v>12</v>
+      </c>
+      <c r="E40" t="s">
+        <v>189</v>
+      </c>
+      <c r="F40" t="s">
+        <v>14</v>
+      </c>
+      <c r="G40" t="s">
+        <v>190</v>
+      </c>
+      <c r="H40" t="s">
+        <v>191</v>
+      </c>
+      <c r="I40" t="s">
+        <v>192</v>
+      </c>
+      <c r="J40" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>194</v>
+      </c>
+      <c r="B41" t="s">
+        <v>12</v>
+      </c>
+      <c r="C41" t="s">
+        <v>12</v>
+      </c>
+      <c r="D41" t="s">
+        <v>12</v>
+      </c>
+      <c r="E41" t="s">
+        <v>195</v>
+      </c>
+      <c r="F41" t="s">
+        <v>14</v>
+      </c>
+      <c r="G41" t="s">
+        <v>184</v>
+      </c>
+      <c r="H41" t="s">
+        <v>196</v>
+      </c>
+      <c r="I41" t="s">
+        <v>197</v>
+      </c>
+      <c r="J41" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>199</v>
+      </c>
+      <c r="B42" t="s">
+        <v>12</v>
+      </c>
+      <c r="C42" t="s">
+        <v>12</v>
+      </c>
+      <c r="D42" t="s">
+        <v>12</v>
+      </c>
+      <c r="E42" t="s">
+        <v>200</v>
+      </c>
+      <c r="F42" t="s">
+        <v>14</v>
+      </c>
+      <c r="G42" t="s">
+        <v>184</v>
+      </c>
+      <c r="H42" t="s">
+        <v>201</v>
+      </c>
+      <c r="I42" t="s">
+        <v>202</v>
+      </c>
+      <c r="J42" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>204</v>
+      </c>
+      <c r="B43" t="s">
+        <v>12</v>
+      </c>
+      <c r="C43" t="s">
+        <v>12</v>
+      </c>
+      <c r="D43" t="s">
+        <v>12</v>
+      </c>
+      <c r="E43" t="s">
+        <v>205</v>
+      </c>
+      <c r="F43" t="s">
+        <v>14</v>
+      </c>
+      <c r="G43" t="s">
+        <v>184</v>
+      </c>
+      <c r="H43" t="s">
+        <v>206</v>
+      </c>
+      <c r="I43" t="s">
+        <v>207</v>
+      </c>
+      <c r="J43" t="s">
+        <v>208</v>
       </c>
     </row>
   </sheetData>

</xml_diff>